<commit_message>
docs: deliver Debian installation recovery guide and executed acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/testing/generated/A-mob-lifetime.xlsx
+++ b/docs/testing/generated/A-mob-lifetime.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="StockLOG" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Full precision" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'StockLOG'!$A$4:$F$16</definedName>
@@ -441,7 +442,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SYNTHETIC ACCEPTANCE FIXTURE. AUD. Animal selection filters never clip lifetime financials. Unknown purchase cost makes P/L incomplete. Active animals show costs/revenue to date, not final realised sale. Timestamps are Unix seconds; property timezone Australia/Melbourne. Stored allocations retain 12 decimal places.</t>
+          <t>SYNTHETIC ACCEPTANCE FIXTURE. AUD. Date/attribute filters select animals; their finances always cover the full lifetime. Unknown purchase prices make P/L incomplete. Active animals show costs/revenue to date, not a final sale outcome. Export dates use your display timezone. Property timezone Australia/Melbourne. Amounts are displayed to cents with reconciliation rounding; Excel also includes full-precision values.</t>
         </is>
       </c>
     </row>
@@ -453,7 +454,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"dataset": "animals", "filters": {"mob": "1"}, "columns": ["animal", "status", "cost", "revenue", "profit", "financial_complete"]}</t>
+          <t>Animals; Mob: April; Attributes: current; Filters: all</t>
         </is>
       </c>
     </row>
@@ -502,17 +503,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>171.500000000000</t>
+          <t>171.50</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0E-12</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>-171.500000000000</t>
+          <t>-171.50</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -534,17 +535,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>171.500000000000</t>
+          <t>171.50</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0E-12</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>-171.500000000000</t>
+          <t>-171.50</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -566,17 +567,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1055.000000000000</t>
+          <t>1055.00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>945.000000000000</t>
+          <t>945.00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -598,17 +599,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1055.000000000000</t>
+          <t>1055.00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>945.000000000000</t>
+          <t>945.00</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -630,17 +631,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1055.000000000000</t>
+          <t>1055.00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>945.000000000000</t>
+          <t>945.00</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -662,17 +663,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1050.000000000000</t>
+          <t>1050.00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>950.000000000000</t>
+          <t>950.00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -694,17 +695,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1050.000000000000</t>
+          <t>1050.00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>950.000000000000</t>
+          <t>950.00</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -726,17 +727,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1050.000000000000</t>
+          <t>1050.00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>950.000000000000</t>
+          <t>950.00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -758,17 +759,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1040.000000000000</t>
+          <t>1040.00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>960.000000000000</t>
+          <t>960.00</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -790,17 +791,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1040.000000000000</t>
+          <t>1040.00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>960.000000000000</t>
+          <t>960.00</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -822,17 +823,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1040.000000000000</t>
+          <t>1040.00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>960.000000000000</t>
+          <t>960.00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -854,17 +855,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1040.000000000000</t>
+          <t>1040.00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2000.000000000000</t>
+          <t>2000.00</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>960.000000000000</t>
+          <t>960.00</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -890,4 +891,441 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Stored precision in AUD/quantities; no financial lifetime clipping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>financial_complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TESTA00000000001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>171.500000000000</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0E-12</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>-171.500000000000</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TESTA00000000002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dead</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>171.500000000000</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0E-12</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-171.500000000000</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TESTA00000000003</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1055.000000000000</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>945.000000000000</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TESTA00000000004</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1055.000000000000</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>945.000000000000</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TESTA00000000005</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1055.000000000000</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>945.000000000000</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TESTA00000000006</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1050.000000000000</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>950.000000000000</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TESTA00000000007</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1050.000000000000</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>950.000000000000</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TESTA00000000008</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1050.000000000000</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>950.000000000000</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TESTA00000000009</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1040.000000000000</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>960.000000000000</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TESTA00000000010</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1040.000000000000</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>960.000000000000</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TESTA00000000011</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1040.000000000000</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>960.000000000000</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TESTA00000000012</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>exited</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1040.000000000000</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2000.000000000000</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>960.000000000000</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>